<commit_message>
Update Zomato reconciliation template (template.xlsx) and cleanup tracked pycache
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Varun\Desktop\Backup AutoRecons\Zomato Auto recons\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Varun\Desktop\Backup AutoRecons\Zomato Auto recons - Copy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7E9493-9301-4147-AD6B-3B5BDC647793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED7D5CE8-8F2D-4E37-B421-8E9A39220AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="882" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="882" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">BANK!$A$10:$G$173</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Cashflow!$A$1:$I$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Cashflow!$A$1:$J$44</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -1507,7 +1507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="40">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -1988,6 +1988,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2002,7 +2015,7 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2297,6 +2310,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2320,7 +2339,12 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2352,13 +2376,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>56744</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>836899</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>90090</xdr:rowOff>
@@ -2407,13 +2431,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>106365</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>120804</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>967840</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>157976</xdr:rowOff>
@@ -2456,13 +2480,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>167640</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>875285</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>115420</xdr:rowOff>
@@ -2505,13 +2529,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>22860</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>137160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>730505</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>46840</xdr:rowOff>
@@ -2870,7 +2894,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:J1007"/>
+  <dimension ref="B1:K1007"/>
   <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4.88671875" style="117" customWidth="1"/>
@@ -2879,42 +2903,46 @@
     <col min="5" max="5" width="12.5546875" style="117" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.109375" style="117" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.88671875" style="117" customWidth="1"/>
-    <col min="8" max="8" width="14" style="117" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="12.5546875" style="117" customWidth="1"/>
-    <col min="11" max="16384" width="12.5546875" style="117"/>
+    <col min="8" max="8" width="12.88671875" style="138" customWidth="1"/>
+    <col min="9" max="9" width="14" style="117" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12.5546875" style="117" customWidth="1"/>
+    <col min="12" max="16384" width="12.5546875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="15" customHeight="1">
-      <c r="B1" s="138"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="E1" s="139"/>
-      <c r="F1" s="139"/>
-      <c r="G1" s="139"/>
-      <c r="H1" s="139"/>
-      <c r="I1" s="6"/>
-    </row>
-    <row r="2" spans="2:9" ht="16.5" customHeight="1">
-      <c r="B2" s="140" t="s">
+    <row r="1" spans="2:10" ht="15" customHeight="1">
+      <c r="B1" s="142"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="143"/>
+      <c r="J1" s="6"/>
+    </row>
+    <row r="2" spans="2:10" ht="16.5" customHeight="1">
+      <c r="B2" s="144" t="s">
         <v>417</v>
       </c>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-    </row>
-    <row r="3" spans="2:9" ht="12" customHeight="1" thickBot="1">
-      <c r="B3" s="141"/>
-      <c r="C3" s="139"/>
-      <c r="D3" s="139"/>
-      <c r="E3" s="139"/>
-      <c r="F3" s="139"/>
-      <c r="G3" s="139"/>
-      <c r="H3" s="139"/>
-    </row>
-    <row r="4" spans="2:9" ht="15" customHeight="1" thickBot="1">
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+    </row>
+    <row r="3" spans="2:10" ht="12" customHeight="1" thickBot="1">
+      <c r="B3" s="145"/>
+      <c r="C3" s="143"/>
+      <c r="D3" s="143"/>
+      <c r="E3" s="143"/>
+      <c r="F3" s="143"/>
+      <c r="G3" s="143"/>
+      <c r="H3" s="143"/>
+      <c r="I3" s="143"/>
+    </row>
+    <row r="4" spans="2:10" ht="15" customHeight="1" thickBot="1">
       <c r="B4" s="13" t="s">
         <v>0</v>
       </c>
@@ -2923,20 +2951,22 @@
       <c r="E4" s="120"/>
       <c r="F4" s="121"/>
       <c r="G4" s="120"/>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="151"/>
+      <c r="I4" s="14" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="12" customHeight="1">
+    <row r="5" spans="2:10" ht="12" customHeight="1">
       <c r="B5" s="15"/>
       <c r="C5" s="16"/>
       <c r="D5" s="17"/>
       <c r="E5" s="16"/>
       <c r="F5" s="17"/>
       <c r="G5" s="18"/>
-      <c r="H5" s="16"/>
-    </row>
-    <row r="6" spans="2:9" ht="12" customHeight="1">
+      <c r="H5" s="18"/>
+      <c r="I5" s="16"/>
+    </row>
+    <row r="6" spans="2:10" ht="12" customHeight="1">
       <c r="B6" s="15" t="s">
         <v>2</v>
       </c>
@@ -2945,21 +2975,23 @@
       <c r="E6" s="15"/>
       <c r="F6" s="15"/>
       <c r="G6" s="99"/>
-      <c r="H6" s="96">
+      <c r="H6" s="99"/>
+      <c r="I6" s="96">
         <f>SUM(C6:G6)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:9" ht="12" customHeight="1">
+    <row r="7" spans="2:10" ht="12" customHeight="1">
       <c r="B7" s="15"/>
       <c r="C7" s="96"/>
       <c r="D7" s="97"/>
       <c r="E7" s="96"/>
       <c r="F7" s="97"/>
       <c r="G7" s="98"/>
-      <c r="H7" s="96"/>
-    </row>
-    <row r="8" spans="2:9" ht="12" customHeight="1">
+      <c r="H7" s="98"/>
+      <c r="I7" s="96"/>
+    </row>
+    <row r="8" spans="2:10" ht="12" customHeight="1">
       <c r="B8" s="15" t="s">
         <v>3</v>
       </c>
@@ -2983,21 +3015,26 @@
         <f>Cashflow!G10</f>
         <v>0</v>
       </c>
-      <c r="H8" s="96">
-        <f>SUM(C8:G8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" ht="12" customHeight="1">
+      <c r="H8" s="99">
+        <f>Cashflow!I10</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="96">
+        <f>SUM(C8:H8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="12" customHeight="1">
       <c r="B9" s="15"/>
       <c r="C9" s="96"/>
       <c r="D9" s="97"/>
       <c r="E9" s="96"/>
       <c r="F9" s="97"/>
       <c r="G9" s="98"/>
-      <c r="H9" s="96"/>
-    </row>
-    <row r="10" spans="2:9" ht="12" customHeight="1">
+      <c r="H9" s="98"/>
+      <c r="I9" s="96"/>
+    </row>
+    <row r="10" spans="2:10" ht="12" customHeight="1">
       <c r="B10" s="19" t="s">
         <v>4</v>
       </c>
@@ -3006,7 +3043,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="137">
-        <f t="shared" ref="D10:H10" si="0">IFERROR(D8/D6,)</f>
+        <f t="shared" ref="D10:I10" si="0">IFERROR(D8/D6,)</f>
         <v>0</v>
       </c>
       <c r="E10" s="137">
@@ -3025,18 +3062,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I10" s="122"/>
-    </row>
-    <row r="11" spans="2:9" ht="12" customHeight="1">
+      <c r="I10" s="137">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="122"/>
+    </row>
+    <row r="11" spans="2:10" ht="12" customHeight="1">
       <c r="B11" s="15"/>
       <c r="C11" s="96"/>
       <c r="D11" s="97"/>
       <c r="E11" s="96"/>
       <c r="F11" s="97"/>
       <c r="G11" s="98"/>
-      <c r="H11" s="96"/>
-    </row>
-    <row r="12" spans="2:9" ht="12" customHeight="1">
+      <c r="H11" s="98"/>
+      <c r="I11" s="96"/>
+    </row>
+    <row r="12" spans="2:10" ht="12" customHeight="1">
       <c r="B12" s="15" t="s">
         <v>5</v>
       </c>
@@ -3056,20 +3098,24 @@
         <v>0</v>
       </c>
       <c r="H12" s="99">
-        <f>SUM(C12:G12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" ht="12" customHeight="1">
+        <v>0</v>
+      </c>
+      <c r="I12" s="99">
+        <f>SUM(C12:H12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="12" customHeight="1">
       <c r="B13" s="15"/>
       <c r="C13" s="99"/>
       <c r="D13" s="101"/>
       <c r="E13" s="99"/>
       <c r="F13" s="101"/>
       <c r="G13" s="102"/>
-      <c r="H13" s="99"/>
-    </row>
-    <row r="14" spans="2:9" ht="12" customHeight="1">
+      <c r="H13" s="102"/>
+      <c r="I13" s="99"/>
+    </row>
+    <row r="14" spans="2:10" ht="12" customHeight="1">
       <c r="B14" s="19" t="s">
         <v>6</v>
       </c>
@@ -3093,21 +3139,26 @@
         <f>Cashflow!G18</f>
         <v>0</v>
       </c>
-      <c r="H14" s="104">
-        <f>SUM(C14:G14)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:9" ht="12" customHeight="1">
+      <c r="H14" s="103">
+        <f>Cashflow!I18</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="104">
+        <f>SUM(C14:H14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="12" customHeight="1">
       <c r="B15" s="15"/>
       <c r="C15" s="99"/>
       <c r="D15" s="101"/>
       <c r="E15" s="99"/>
       <c r="F15" s="101"/>
       <c r="G15" s="102"/>
-      <c r="H15" s="99"/>
-    </row>
-    <row r="16" spans="2:9" ht="14.4" customHeight="1">
+      <c r="H15" s="152"/>
+      <c r="I15" s="99"/>
+    </row>
+    <row r="16" spans="2:10" ht="14.4" customHeight="1">
       <c r="B16" s="15" t="s">
         <v>7</v>
       </c>
@@ -3131,12 +3182,16 @@
         <f>Cashflow!G8</f>
         <v>0</v>
       </c>
-      <c r="H16" s="96">
-        <f>SUM(C16:G16)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" ht="15" customHeight="1">
+      <c r="H16" s="99">
+        <f>Cashflow!I8</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="96">
+        <f>SUM(C16:H16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="15" customHeight="1">
       <c r="B17" s="15"/>
       <c r="C17" s="20">
         <f>IFERROR(C16/C8,)</f>
@@ -3155,21 +3210,26 @@
         <v>0</v>
       </c>
       <c r="G17" s="20">
-        <f t="shared" ref="G17" si="3">IFERROR(G16/G8,)</f>
+        <f t="shared" ref="G17:H17" si="3">IFERROR(G16/G8,)</f>
         <v>0</v>
       </c>
       <c r="H17" s="20">
-        <f t="shared" ref="H17" si="4">IFERROR(H16/H8,)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" ht="15" customHeight="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I17" s="20">
+        <f t="shared" ref="I17" si="4">IFERROR(I16/I8,)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="15" customHeight="1">
       <c r="B18" s="115"/>
       <c r="D18" s="115"/>
       <c r="F18" s="115"/>
       <c r="H18" s="115"/>
-    </row>
-    <row r="19" spans="2:10" ht="12" customHeight="1">
+      <c r="I18" s="115"/>
+    </row>
+    <row r="19" spans="2:11" ht="12" customHeight="1">
       <c r="B19" s="15" t="s">
         <v>8</v>
       </c>
@@ -3178,12 +3238,13 @@
       <c r="E19" s="116"/>
       <c r="F19" s="116"/>
       <c r="G19" s="116"/>
-      <c r="H19" s="104">
-        <f>SUM(C19:G19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" ht="17.399999999999999" customHeight="1">
+      <c r="H19" s="116"/>
+      <c r="I19" s="104">
+        <f>SUM(C19:H19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="17.399999999999999" customHeight="1">
       <c r="B20" s="25" t="s">
         <v>9</v>
       </c>
@@ -3207,13 +3268,17 @@
         <f>Cashflow!G11</f>
         <v>0</v>
       </c>
-      <c r="H20" s="96">
-        <f>SUM(C20:G20)</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="2"/>
-    </row>
-    <row r="21" spans="2:10" ht="19.2" customHeight="1">
+      <c r="H20" s="105">
+        <f>Cashflow!I11</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="96">
+        <f>SUM(C20:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="2:11" ht="19.2" customHeight="1">
       <c r="B21" s="19" t="s">
         <v>10</v>
       </c>
@@ -3222,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="26">
-        <f t="shared" ref="D21:H21" si="5">IFERROR(D20/D19,)</f>
+        <f t="shared" ref="D21:I21" si="5">IFERROR(D20/D19,)</f>
         <v>0</v>
       </c>
       <c r="E21" s="26">
@@ -3241,19 +3306,24 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J21" s="3"/>
-    </row>
-    <row r="22" spans="2:10" ht="12" customHeight="1">
+      <c r="I21" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="2:11" ht="12" customHeight="1">
       <c r="B22" s="15"/>
       <c r="C22" s="123"/>
       <c r="D22" s="124"/>
       <c r="E22" s="123"/>
       <c r="F22" s="124"/>
       <c r="G22" s="125"/>
-      <c r="H22" s="123"/>
-      <c r="J22" s="3"/>
-    </row>
-    <row r="23" spans="2:10" ht="12" customHeight="1">
+      <c r="H22" s="125"/>
+      <c r="I22" s="123"/>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="2:11" ht="12" customHeight="1">
       <c r="B23" s="19" t="s">
         <v>11</v>
       </c>
@@ -3277,19 +3347,23 @@
         <f>Cashflow!G21</f>
         <v>0</v>
       </c>
-      <c r="H23" s="95">
-        <f>SUM(C23:G23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="2:10" ht="13.8" customHeight="1">
+      <c r="H23" s="103">
+        <f>Cashflow!I21</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="95">
+        <f>SUM(C23:H23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="13.8" customHeight="1">
       <c r="B24" s="15"/>
       <c r="C24" s="21">
         <f>IFERROR(C23/C8,)</f>
         <v>0</v>
       </c>
       <c r="D24" s="21">
-        <f t="shared" ref="D24:H24" si="6">IFERROR(D23/D8,)</f>
+        <f t="shared" ref="D24:I24" si="6">IFERROR(D23/D8,)</f>
         <v>0</v>
       </c>
       <c r="E24" s="21">
@@ -3305,29 +3379,35 @@
         <v>0</v>
       </c>
       <c r="H24" s="21">
+        <f t="shared" ref="H24" si="7">IFERROR(H23/H8,)</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="12" customHeight="1">
+    <row r="25" spans="2:11" ht="12" customHeight="1">
       <c r="B25" s="15"/>
       <c r="C25" s="22"/>
       <c r="D25" s="23"/>
       <c r="E25" s="22"/>
       <c r="F25" s="23"/>
       <c r="G25" s="24"/>
-      <c r="H25" s="22"/>
-    </row>
-    <row r="26" spans="2:10" ht="8.4" customHeight="1">
+      <c r="H25" s="24"/>
+      <c r="I25" s="22"/>
+    </row>
+    <row r="26" spans="2:11" ht="8.4" customHeight="1">
       <c r="B26" s="15"/>
       <c r="C26" s="27"/>
       <c r="D26" s="28"/>
       <c r="E26" s="29"/>
       <c r="F26" s="28"/>
       <c r="G26" s="27"/>
-      <c r="H26" s="22"/>
-    </row>
-    <row r="27" spans="2:10" ht="15" customHeight="1">
+      <c r="H26" s="27"/>
+      <c r="I26" s="22"/>
+    </row>
+    <row r="27" spans="2:11" ht="15" customHeight="1">
       <c r="B27" s="30" t="s">
         <v>12</v>
       </c>
@@ -3351,66 +3431,77 @@
         <f>Cashflow!G13+Cashflow!G26</f>
         <v>0</v>
       </c>
-      <c r="H27" s="110">
-        <f>SUM(C27:G27)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="2:10" ht="15.6" customHeight="1">
+      <c r="H27" s="108">
+        <f>Cashflow!I13+Cashflow!I26</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="110">
+        <f>SUM(C27:H27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="15.6" customHeight="1">
       <c r="B28" s="15"/>
       <c r="C28" s="31">
         <f>IFERROR(C27/C8,)</f>
         <v>0</v>
       </c>
       <c r="D28" s="31">
-        <f t="shared" ref="D28:H28" si="7">IFERROR(D27/D8,)</f>
+        <f t="shared" ref="D28:I28" si="8">IFERROR(D27/D8,)</f>
         <v>0</v>
       </c>
       <c r="E28" s="31">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F28" s="31">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="G28" s="31">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H28" s="31">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="2:10" ht="3" customHeight="1">
+        <f t="shared" ref="H28" si="9">IFERROR(H27/H8,)</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="31">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" ht="3" customHeight="1">
       <c r="B29" s="15"/>
       <c r="C29" s="31"/>
       <c r="D29" s="32"/>
       <c r="E29" s="31"/>
       <c r="F29" s="32"/>
       <c r="G29" s="31"/>
-      <c r="H29" s="21"/>
-    </row>
-    <row r="30" spans="2:10" ht="12" customHeight="1">
+      <c r="H29" s="31"/>
+      <c r="I29" s="21"/>
+    </row>
+    <row r="30" spans="2:11" ht="12" customHeight="1">
       <c r="B30" s="15"/>
       <c r="C30" s="126"/>
       <c r="D30" s="124"/>
       <c r="E30" s="126"/>
       <c r="F30" s="124"/>
       <c r="G30" s="125"/>
-      <c r="H30" s="123"/>
-    </row>
-    <row r="31" spans="2:10" s="136" customFormat="1" ht="12" customHeight="1">
+      <c r="H30" s="125"/>
+      <c r="I30" s="123"/>
+    </row>
+    <row r="31" spans="2:11" s="136" customFormat="1" ht="12" customHeight="1">
       <c r="B31" s="15"/>
       <c r="C31" s="126"/>
       <c r="D31" s="124"/>
       <c r="E31" s="126"/>
       <c r="F31" s="124"/>
       <c r="G31" s="125"/>
-      <c r="H31" s="123"/>
-    </row>
-    <row r="32" spans="2:10" ht="12" customHeight="1">
+      <c r="H31" s="125"/>
+      <c r="I31" s="123"/>
+    </row>
+    <row r="32" spans="2:11" ht="12" customHeight="1">
       <c r="B32" s="15" t="s">
         <v>13</v>
       </c>
@@ -3435,11 +3526,15 @@
         <v>0</v>
       </c>
       <c r="H32" s="96">
-        <f>SUM(C32:G32)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="2:10" ht="2.4" customHeight="1">
+        <f>Cashflow!I36</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="96">
+        <f>SUM(C32:H32)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" ht="2.4" customHeight="1">
       <c r="B33" s="15"/>
       <c r="C33" s="96"/>
       <c r="D33" s="114"/>
@@ -3447,17 +3542,19 @@
       <c r="F33" s="114"/>
       <c r="G33" s="96"/>
       <c r="H33" s="96"/>
-    </row>
-    <row r="34" spans="2:10" ht="12" customHeight="1">
+      <c r="I33" s="96"/>
+    </row>
+    <row r="34" spans="2:11" ht="12" customHeight="1">
       <c r="B34" s="15"/>
       <c r="C34" s="96"/>
       <c r="D34" s="97"/>
       <c r="E34" s="96"/>
       <c r="F34" s="97"/>
       <c r="G34" s="98"/>
-      <c r="H34" s="99"/>
-    </row>
-    <row r="35" spans="2:10" ht="12" customHeight="1">
+      <c r="H34" s="98"/>
+      <c r="I34" s="99"/>
+    </row>
+    <row r="35" spans="2:11" ht="12" customHeight="1">
       <c r="B35" s="15" t="s">
         <v>15</v>
       </c>
@@ -3482,12 +3579,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="96">
-        <f>SUM(C35:G35)</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="4"/>
-    </row>
-    <row r="36" spans="2:10" ht="17.25" customHeight="1" thickBot="1">
+        <f>H8-H14-H20-H23-H27-H32</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="96">
+        <f>SUM(C35:H35)</f>
+        <v>0</v>
+      </c>
+      <c r="K35" s="4"/>
+    </row>
+    <row r="36" spans="2:11" ht="17.25" customHeight="1" thickBot="1">
       <c r="B36" s="33"/>
       <c r="C36" s="34">
         <f>IFERROR(C35/$C$8,)</f>
@@ -3513,42 +3614,46 @@
         <f>IFERROR(H35/H8,)</f>
         <v>0</v>
       </c>
-      <c r="J36" s="4"/>
-    </row>
-    <row r="37" spans="2:10" ht="12" customHeight="1">
+      <c r="I36" s="34">
+        <f>IFERROR(I35/I8,)</f>
+        <v>0</v>
+      </c>
+      <c r="K36" s="4"/>
+    </row>
+    <row r="37" spans="2:11" ht="12" customHeight="1">
       <c r="B37" s="5"/>
     </row>
-    <row r="38" spans="2:10" ht="12" customHeight="1">
+    <row r="38" spans="2:11" ht="12" customHeight="1">
       <c r="B38" s="9"/>
     </row>
-    <row r="39" spans="2:10" ht="12" customHeight="1">
+    <row r="39" spans="2:11" ht="12" customHeight="1">
       <c r="B39" s="10"/>
       <c r="C39" s="1"/>
     </row>
-    <row r="40" spans="2:10" ht="12" customHeight="1">
+    <row r="40" spans="2:11" ht="12" customHeight="1">
       <c r="B40" s="10"/>
       <c r="C40" s="4"/>
     </row>
-    <row r="41" spans="2:10" ht="12" customHeight="1"/>
-    <row r="42" spans="2:10" ht="12" customHeight="1">
+    <row r="41" spans="2:11" ht="12" customHeight="1"/>
+    <row r="42" spans="2:11" ht="12" customHeight="1">
       <c r="B42" s="5"/>
     </row>
-    <row r="43" spans="2:10" ht="12" customHeight="1">
+    <row r="43" spans="2:11" ht="12" customHeight="1">
       <c r="B43" s="5"/>
     </row>
-    <row r="44" spans="2:10" ht="12" customHeight="1">
+    <row r="44" spans="2:11" ht="12" customHeight="1">
       <c r="B44" s="5"/>
     </row>
-    <row r="45" spans="2:10" ht="12" customHeight="1">
+    <row r="45" spans="2:11" ht="12" customHeight="1">
       <c r="B45" s="5"/>
     </row>
-    <row r="46" spans="2:10" ht="12" customHeight="1">
+    <row r="46" spans="2:11" ht="12" customHeight="1">
       <c r="B46" s="5"/>
     </row>
-    <row r="47" spans="2:10" ht="12" customHeight="1">
+    <row r="47" spans="2:11" ht="12" customHeight="1">
       <c r="B47" s="5"/>
     </row>
-    <row r="48" spans="2:10" ht="12" customHeight="1">
+    <row r="48" spans="2:11" ht="12" customHeight="1">
       <c r="B48" s="5"/>
     </row>
     <row r="49" spans="2:2" ht="12" customHeight="1">
@@ -4888,9 +4993,9 @@
     <row r="1007" ht="13.8" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B3:I3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="90" orientation="landscape" r:id="rId1"/>
@@ -4903,55 +5008,58 @@
   <sheetPr codeName="Sheet2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5.21875" style="118" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37" style="118" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.6640625" style="118" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="15.77734375" style="127" customWidth="1"/>
     <col min="5" max="7" width="15.77734375" style="128" customWidth="1"/>
-    <col min="8" max="8" width="15.77734375" style="118" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" style="117" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="11.21875" style="117" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.44140625" style="117" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" style="117" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.109375" style="117" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.44140625" style="117" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" style="117" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="8.88671875" style="117" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="117"/>
+    <col min="8" max="8" width="15.77734375" style="140" customWidth="1"/>
+    <col min="9" max="9" width="15.77734375" style="118" customWidth="1"/>
+    <col min="10" max="10" width="12.109375" style="117" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.21875" style="117" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.44140625" style="117" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.109375" style="117" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.109375" style="117" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.44140625" style="117" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.109375" style="117" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="8.88671875" style="117" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="18" customHeight="1">
-      <c r="A1" s="146">
+    <row r="1" spans="1:18" ht="18" customHeight="1">
+      <c r="A1" s="150">
         <f>Summary!B1</f>
         <v>0</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="E1" s="145"/>
-      <c r="F1" s="145"/>
-      <c r="G1" s="145"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="7"/>
+      <c r="B1" s="147"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="147"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
-    </row>
-    <row r="2" spans="1:17" ht="15.6" customHeight="1">
-      <c r="A2" s="142" t="s">
+      <c r="M1" s="7"/>
+    </row>
+    <row r="2" spans="1:18" ht="15.6" customHeight="1">
+      <c r="A2" s="146" t="s">
         <v>414</v>
       </c>
-      <c r="B2" s="143"/>
-      <c r="C2" s="144"/>
-      <c r="D2" s="144"/>
-      <c r="E2" s="145"/>
-      <c r="F2" s="145"/>
-      <c r="G2" s="145"/>
-      <c r="H2" s="143"/>
-    </row>
-    <row r="3" spans="1:17" ht="15" customHeight="1" thickBot="1">
+      <c r="B2" s="147"/>
+      <c r="C2" s="148"/>
+      <c r="D2" s="148"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="147"/>
+    </row>
+    <row r="3" spans="1:18" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="46"/>
       <c r="B3" s="46"/>
       <c r="C3" s="46"/>
@@ -4960,8 +5068,9 @@
       <c r="F3" s="46"/>
       <c r="G3" s="46"/>
       <c r="H3" s="46"/>
-    </row>
-    <row r="4" spans="1:17" ht="15" customHeight="1" thickBot="1">
+      <c r="I3" s="46"/>
+    </row>
+    <row r="4" spans="1:18" ht="15" customHeight="1" thickBot="1">
       <c r="A4" s="59" t="s">
         <v>16</v>
       </c>
@@ -4988,11 +5097,15 @@
         <f>Summary!G4</f>
         <v>0</v>
       </c>
-      <c r="H4" s="61" t="s">
+      <c r="H4" s="61">
+        <f>Summary!H4</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="61" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:18">
       <c r="A5" s="111">
         <v>1</v>
       </c>
@@ -5004,14 +5117,15 @@
       <c r="E5" s="88"/>
       <c r="F5" s="64"/>
       <c r="G5" s="64"/>
-      <c r="H5" s="88">
-        <f>SUM(C5:G5)</f>
-        <v>0</v>
-      </c>
-      <c r="I5" s="122"/>
+      <c r="H5" s="88"/>
+      <c r="I5" s="88">
+        <f>SUM(C5:H5)</f>
+        <v>0</v>
+      </c>
       <c r="J5" s="122"/>
-    </row>
-    <row r="6" spans="1:17">
+      <c r="K5" s="122"/>
+    </row>
+    <row r="6" spans="1:18">
       <c r="A6" s="112"/>
       <c r="B6" s="62" t="s">
         <v>18</v>
@@ -5021,14 +5135,15 @@
       <c r="E6" s="62"/>
       <c r="F6" s="62"/>
       <c r="G6" s="88"/>
-      <c r="H6" s="88">
-        <f>SUM(C6:G6)</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="122"/>
-      <c r="K6" s="122"/>
-    </row>
-    <row r="7" spans="1:17">
+      <c r="H6" s="88"/>
+      <c r="I6" s="88">
+        <f>SUM(C6:H6)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="122"/>
+      <c r="L6" s="122"/>
+    </row>
+    <row r="7" spans="1:18">
       <c r="A7" s="112"/>
       <c r="B7" s="62" t="s">
         <v>19</v>
@@ -5038,17 +5153,18 @@
       <c r="E7" s="88"/>
       <c r="F7" s="88"/>
       <c r="G7" s="88"/>
-      <c r="H7" s="88">
-        <f>SUM(C7:G7)</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="122"/>
+      <c r="H7" s="88"/>
+      <c r="I7" s="88">
+        <f>SUM(C7:H7)</f>
+        <v>0</v>
+      </c>
       <c r="J7" s="122"/>
       <c r="K7" s="122"/>
       <c r="L7" s="122"/>
       <c r="M7" s="122"/>
-    </row>
-    <row r="8" spans="1:17">
+      <c r="N7" s="122"/>
+    </row>
+    <row r="8" spans="1:18">
       <c r="A8" s="112"/>
       <c r="B8" s="62" t="s">
         <v>20</v>
@@ -5058,11 +5174,11 @@
       <c r="E8" s="88"/>
       <c r="F8" s="88"/>
       <c r="G8" s="88"/>
-      <c r="H8" s="88">
-        <f>SUM(C8:G8)</f>
-        <v>0</v>
-      </c>
-      <c r="I8" s="122"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88">
+        <f>SUM(C8:H8)</f>
+        <v>0</v>
+      </c>
       <c r="J8" s="122"/>
       <c r="K8" s="122"/>
       <c r="L8" s="122"/>
@@ -5070,8 +5186,9 @@
       <c r="N8" s="122"/>
       <c r="O8" s="122"/>
       <c r="P8" s="122"/>
-    </row>
-    <row r="9" spans="1:17">
+      <c r="Q8" s="122"/>
+    </row>
+    <row r="9" spans="1:18">
       <c r="A9" s="112"/>
       <c r="B9" s="62" t="s">
         <v>21</v>
@@ -5081,20 +5198,21 @@
       <c r="E9" s="88"/>
       <c r="F9" s="88"/>
       <c r="G9" s="88"/>
-      <c r="H9" s="88">
-        <f>SUM(C9:G9)</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="122"/>
-      <c r="M9" s="117" t="s">
+      <c r="H9" s="88"/>
+      <c r="I9" s="88">
+        <f>SUM(C9:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="11"/>
+      <c r="K9" s="122"/>
+      <c r="N9" s="117" t="s">
         <v>22</v>
       </c>
-      <c r="N9" s="117" t="s">
+      <c r="O9" s="117" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:18">
       <c r="A10" s="112"/>
       <c r="B10" s="66" t="s">
         <v>24</v>
@@ -5104,7 +5222,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="67">
-        <f t="shared" ref="D10:H10" si="0">D5+D6+D9+D7-D8</f>
+        <f t="shared" ref="D10:I10" si="0">D5+D6+D9+D7-D8</f>
         <v>0</v>
       </c>
       <c r="E10" s="68">
@@ -5120,21 +5238,25 @@
         <v>0</v>
       </c>
       <c r="H10" s="68">
+        <f>H5+H6+H9+H7-H8</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="68">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I10" s="122"/>
-      <c r="J10" s="1"/>
-      <c r="M10" s="1">
-        <f>H10-H29</f>
-        <v>0</v>
-      </c>
-      <c r="N10" s="117">
-        <f>H12*100/118</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" ht="15" customHeight="1" thickBot="1">
+      <c r="J10" s="122"/>
+      <c r="K10" s="1"/>
+      <c r="N10" s="1">
+        <f>I10-I29</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="117">
+        <f>I12*100/118</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15" customHeight="1" thickBot="1">
       <c r="A11" s="111">
         <v>2</v>
       </c>
@@ -5142,7 +5264,7 @@
         <v>25</v>
       </c>
       <c r="C11" s="70">
-        <f t="shared" ref="C11:H11" si="1">C12</f>
+        <f t="shared" ref="C11:I11" si="1">C12</f>
         <v>0</v>
       </c>
       <c r="D11" s="70">
@@ -5165,10 +5287,14 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="1"/>
-    </row>
-    <row r="12" spans="1:17">
+      <c r="I11" s="70">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="1:18">
       <c r="A12" s="113"/>
       <c r="B12" s="71" t="s">
         <v>26</v>
@@ -5178,15 +5304,16 @@
       <c r="E12" s="73"/>
       <c r="F12" s="74"/>
       <c r="G12" s="74"/>
-      <c r="H12" s="74">
-        <f>SUM(C12:G12)</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="122"/>
+      <c r="H12" s="74"/>
+      <c r="I12" s="74">
+        <f>SUM(C12:H12)</f>
+        <v>0</v>
+      </c>
       <c r="J12" s="122"/>
       <c r="K12" s="122"/>
-    </row>
-    <row r="13" spans="1:17">
+      <c r="L12" s="122"/>
+    </row>
+    <row r="13" spans="1:18">
       <c r="A13" s="111">
         <v>3</v>
       </c>
@@ -5198,7 +5325,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="67">
-        <f t="shared" ref="D13:H13" si="2">D14+D16-D15+D17</f>
+        <f t="shared" ref="D13:I13" si="2">D14+D16-D15+D17</f>
         <v>0</v>
       </c>
       <c r="E13" s="67">
@@ -5217,8 +5344,12 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:17">
+      <c r="I13" s="67">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18">
       <c r="A14" s="113"/>
       <c r="B14" s="75" t="s">
         <v>28</v>
@@ -5228,16 +5359,17 @@
       <c r="E14" s="77"/>
       <c r="F14" s="78"/>
       <c r="G14" s="78"/>
-      <c r="H14" s="78">
-        <f>SUM(C14:G14)</f>
-        <v>0</v>
-      </c>
-      <c r="I14" s="122"/>
+      <c r="H14" s="78"/>
+      <c r="I14" s="78">
+        <f>SUM(C14:H14)</f>
+        <v>0</v>
+      </c>
       <c r="J14" s="122"/>
       <c r="K14" s="122"/>
       <c r="L14" s="122"/>
-    </row>
-    <row r="15" spans="1:17">
+      <c r="M14" s="122"/>
+    </row>
+    <row r="15" spans="1:18">
       <c r="A15" s="113"/>
       <c r="B15" s="79" t="s">
         <v>29</v>
@@ -5247,38 +5379,39 @@
       <c r="E15" s="78"/>
       <c r="F15" s="78"/>
       <c r="G15" s="77"/>
-      <c r="H15" s="78">
-        <f>SUM(C15:G15)</f>
-        <v>0</v>
-      </c>
-      <c r="I15" s="122"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78">
+        <f>SUM(C15:H15)</f>
+        <v>0</v>
+      </c>
       <c r="J15" s="122"/>
       <c r="K15" s="122"/>
-      <c r="L15" s="122" t="s">
+      <c r="L15" s="122"/>
+      <c r="M15" s="122" t="s">
         <v>30</v>
       </c>
-      <c r="M15" s="1">
+      <c r="N15" s="1">
         <f>C10+C8-C29</f>
         <v>0</v>
       </c>
-      <c r="N15" s="1">
+      <c r="O15" s="1">
         <f>D10+D8-D29</f>
         <v>0</v>
       </c>
-      <c r="O15" s="1">
+      <c r="P15" s="1">
         <f>E10+E8-E29</f>
         <v>0</v>
       </c>
-      <c r="P15" s="1">
+      <c r="Q15" s="1">
         <f>F10+F8-F29</f>
         <v>0</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="R15" s="1">
         <f>G10+G8-G29</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:18">
       <c r="A16" s="112"/>
       <c r="B16" s="62" t="s">
         <v>31</v>
@@ -5288,35 +5421,36 @@
       <c r="E16" s="81"/>
       <c r="F16" s="81"/>
       <c r="G16" s="88"/>
-      <c r="H16" s="88">
-        <f>SUM(C16:G16)</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="122" t="s">
+      <c r="H16" s="88"/>
+      <c r="I16" s="88">
+        <f>SUM(C16:H16)</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="122" t="s">
         <v>32</v>
       </c>
-      <c r="M16" s="1">
+      <c r="N16" s="1">
         <f>C8</f>
         <v>0</v>
       </c>
-      <c r="N16" s="1">
+      <c r="O16" s="1">
         <f>D8</f>
         <v>0</v>
       </c>
-      <c r="O16" s="1">
+      <c r="P16" s="1">
         <f>E8</f>
         <v>0</v>
       </c>
-      <c r="P16" s="1">
+      <c r="Q16" s="1">
         <f>F8</f>
         <v>0</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="R16" s="1">
         <f>G8</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:18">
       <c r="A17" s="111">
         <v>4</v>
       </c>
@@ -5338,35 +5472,36 @@
       <c r="G17" s="88">
         <v>0</v>
       </c>
-      <c r="H17" s="88">
-        <f>SUM(C17:G17)</f>
-        <v>0</v>
-      </c>
-      <c r="L17" s="117" t="s">
+      <c r="H17" s="88"/>
+      <c r="I17" s="88">
+        <f>SUM(C17:H17)</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="117" t="s">
         <v>34</v>
       </c>
-      <c r="M17" s="1">
+      <c r="N17" s="1">
         <f>C12-C15</f>
         <v>0</v>
       </c>
-      <c r="N17" s="1">
+      <c r="O17" s="1">
         <f>D12-D15</f>
         <v>0</v>
       </c>
-      <c r="O17" s="1">
+      <c r="P17" s="1">
         <f>E12-E15</f>
         <v>0</v>
       </c>
-      <c r="P17" s="1">
+      <c r="Q17" s="1">
         <f>F12-F15</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="R17" s="1">
         <f>G12-G15</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="14.4" customHeight="1">
+    <row r="18" spans="1:18" ht="14.4" customHeight="1">
       <c r="A18" s="112"/>
       <c r="B18" s="66" t="s">
         <v>35</v>
@@ -5391,36 +5526,40 @@
         <f>SUM(G19:G20)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="68">
-        <f>H19+H20</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="122"/>
-      <c r="L18" s="122" t="s">
+      <c r="H18" s="67">
+        <f>SUM(H19:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="68">
+        <f>I19+I20</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="122"/>
+      <c r="M18" s="122" t="s">
         <v>36</v>
       </c>
-      <c r="M18" s="1">
+      <c r="N18" s="1">
         <f>C27</f>
         <v>0</v>
       </c>
-      <c r="N18" s="1">
+      <c r="O18" s="1">
         <f>D27</f>
         <v>0</v>
       </c>
-      <c r="O18" s="1">
+      <c r="P18" s="1">
         <f>E27</f>
         <v>0</v>
       </c>
-      <c r="P18" s="1">
+      <c r="Q18" s="1">
         <f>F27</f>
         <v>0</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="R18" s="1">
         <f>G27</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:18">
       <c r="A19" s="111"/>
       <c r="B19" s="62" t="s">
         <v>37</v>
@@ -5430,35 +5569,36 @@
       <c r="E19" s="88"/>
       <c r="F19" s="88"/>
       <c r="G19" s="88"/>
-      <c r="H19" s="88">
-        <f>SUM(C19:G19)</f>
-        <v>0</v>
-      </c>
-      <c r="L19" s="129" t="s">
+      <c r="H19" s="88"/>
+      <c r="I19" s="88">
+        <f>SUM(C19:H19)</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="129" t="s">
         <v>38</v>
       </c>
-      <c r="M19" s="1">
+      <c r="N19" s="1">
         <f>C14</f>
         <v>0</v>
       </c>
-      <c r="N19" s="1">
+      <c r="O19" s="1">
         <f>D14</f>
         <v>0</v>
       </c>
-      <c r="O19" s="1">
+      <c r="P19" s="1">
         <f>E14</f>
         <v>0</v>
       </c>
-      <c r="P19" s="1">
+      <c r="Q19" s="1">
         <f>F14</f>
         <v>0</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="R19" s="1">
         <f>G14</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:18">
       <c r="A20" s="111">
         <v>5</v>
       </c>
@@ -5481,40 +5621,43 @@
         <v>0</v>
       </c>
       <c r="H20" s="88">
-        <f>SUM(C20:G20)</f>
-        <v>0</v>
-      </c>
-      <c r="L20" s="117" t="s">
+        <v>0</v>
+      </c>
+      <c r="I20" s="88">
+        <f>SUM(C20:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="M20" s="117" t="s">
         <v>40</v>
       </c>
-      <c r="M20" s="1">
+      <c r="N20" s="1">
         <f>C16</f>
         <v>0</v>
       </c>
-      <c r="N20" s="1">
+      <c r="O20" s="1">
         <f>D16</f>
         <v>0</v>
       </c>
-      <c r="O20" s="1">
+      <c r="P20" s="1">
         <f>E16</f>
         <v>0</v>
       </c>
-      <c r="P20" s="1">
+      <c r="Q20" s="1">
         <f>F16</f>
         <v>0</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="R20" s="1">
         <f>G16</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="17.399999999999999" customHeight="1">
+    <row r="21" spans="1:18" ht="17.399999999999999" customHeight="1">
       <c r="A21" s="112"/>
       <c r="B21" s="66" t="s">
         <v>41</v>
       </c>
       <c r="C21" s="67">
-        <f t="shared" ref="C21:H21" si="3">C22+C23+C24</f>
+        <f t="shared" ref="C21:I21" si="3">C22+C23+C24</f>
         <v>0</v>
       </c>
       <c r="D21" s="67">
@@ -5537,31 +5680,35 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L21" s="117" t="s">
+      <c r="I21" s="68">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M21" s="117" t="s">
         <v>42</v>
       </c>
-      <c r="M21" s="117">
+      <c r="N21" s="117">
         <f>(C12*100/118)*2%</f>
         <v>0</v>
       </c>
-      <c r="N21" s="117">
+      <c r="O21" s="117">
         <f>(D12*100/118)*2%</f>
         <v>0</v>
       </c>
-      <c r="O21" s="117">
+      <c r="P21" s="117">
         <f>(E12*100/118)*2%</f>
         <v>0</v>
       </c>
-      <c r="P21" s="117">
+      <c r="Q21" s="117">
         <f>(F12*100/118)*2%</f>
         <v>0</v>
       </c>
-      <c r="Q21" s="117">
+      <c r="R21" s="117">
         <f>(G12*100/118)*2%</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="19.2" customHeight="1">
+    <row r="22" spans="1:18" ht="19.2" customHeight="1">
       <c r="A22" s="112"/>
       <c r="B22" s="62" t="s">
         <v>43</v>
@@ -5582,13 +5729,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="88">
-        <f>SUM(C22:G22)</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="130"/>
+        <v>0</v>
+      </c>
+      <c r="I22" s="88">
+        <f>SUM(C22:H22)</f>
+        <v>0</v>
+      </c>
       <c r="K22" s="130"/>
-    </row>
-    <row r="23" spans="1:17">
+      <c r="L22" s="130"/>
+    </row>
+    <row r="23" spans="1:18">
       <c r="A23" s="112"/>
       <c r="B23" s="62" t="s">
         <v>44</v>
@@ -5609,11 +5759,14 @@
         <v>0</v>
       </c>
       <c r="H23" s="88">
-        <f>SUM(C23:G23)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17">
+        <v>0</v>
+      </c>
+      <c r="I23" s="88">
+        <f>SUM(C23:H23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18">
       <c r="A24" s="112"/>
       <c r="B24" s="62" t="s">
         <v>45</v>
@@ -5634,12 +5787,15 @@
         <v>0</v>
       </c>
       <c r="H24" s="88">
-        <f>SUM(C24:G24)</f>
-        <v>0</v>
-      </c>
-      <c r="M24" s="122"/>
-    </row>
-    <row r="25" spans="1:17">
+        <v>0</v>
+      </c>
+      <c r="I24" s="88">
+        <f>SUM(C24:H24)</f>
+        <v>0</v>
+      </c>
+      <c r="N24" s="122"/>
+    </row>
+    <row r="25" spans="1:18">
       <c r="A25" s="111">
         <v>6</v>
       </c>
@@ -5647,61 +5803,69 @@
         <v>46</v>
       </c>
       <c r="C25" s="67">
-        <f>C10-C11-C18-C21-C13-C29</f>
+        <f t="shared" ref="C25:I25" si="4">C10-C11-C18-C21-C13-C29</f>
         <v>0</v>
       </c>
       <c r="D25" s="67">
-        <f>D10-D11-D18-D21-D13-D29</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="E25" s="67">
-        <f>E10-E11-E18-E21-E13-E29</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="F25" s="67">
-        <f>F10-F11-F18-F21-F13-F29</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G25" s="67">
-        <f>G10-G11-G18-G21-G13-G29</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H25" s="67">
-        <f>H10-H11-H18-H21-H13-H29</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17">
+        <f t="shared" ref="H25" si="5">H10-H11-H18-H21-H13-H29</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="67">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18">
       <c r="A26" s="112"/>
       <c r="B26" s="66" t="s">
         <v>47</v>
       </c>
       <c r="C26" s="67">
-        <f t="shared" ref="C26:H26" si="4">SUM(C27:C29)</f>
+        <f t="shared" ref="C26:I26" si="6">SUM(C27:C29)</f>
         <v>0</v>
       </c>
       <c r="D26" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="E26" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="F26" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="G26" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H26" s="67">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17">
+        <f t="shared" ref="H26" si="7">SUM(H27:H29)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="67">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18">
       <c r="A27" s="112"/>
       <c r="B27" s="62" t="s">
         <v>48</v>
@@ -5711,12 +5875,13 @@
       <c r="E27" s="82"/>
       <c r="F27" s="88"/>
       <c r="G27" s="88"/>
-      <c r="H27" s="88">
-        <f>SUM(C27:G27)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" ht="15" customHeight="1">
+      <c r="H27" s="88"/>
+      <c r="I27" s="88">
+        <f>SUM(C27:H27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="15" customHeight="1">
       <c r="A28" s="112"/>
       <c r="B28" s="62" t="s">
         <v>49</v>
@@ -5726,12 +5891,13 @@
       <c r="E28" s="88"/>
       <c r="F28" s="82"/>
       <c r="G28" s="88"/>
-      <c r="H28" s="88">
-        <f>SUM(C28:G28)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" ht="15.6" customHeight="1">
+      <c r="H28" s="88"/>
+      <c r="I28" s="88">
+        <f>SUM(C28:H28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="15.6" customHeight="1">
       <c r="A29" s="111">
         <v>7</v>
       </c>
@@ -5743,12 +5909,13 @@
       <c r="E29" s="88"/>
       <c r="F29" s="88"/>
       <c r="G29" s="88"/>
-      <c r="H29" s="88">
-        <f>SUM(C29:G29)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17">
+      <c r="H29" s="88"/>
+      <c r="I29" s="88">
+        <f>SUM(C29:H29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18">
       <c r="A30" s="111"/>
       <c r="B30" s="66" t="s">
         <v>51</v>
@@ -5758,28 +5925,32 @@
         <v>0</v>
       </c>
       <c r="D30" s="67">
-        <f t="shared" ref="D30:H30" si="5">D25-D27-D28-D34</f>
+        <f t="shared" ref="D30:I30" si="8">D25-D27-D28-D34</f>
         <v>0</v>
       </c>
       <c r="E30" s="67">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F30" s="67">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="G30" s="67">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H30" s="67">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J30" s="122"/>
-    </row>
-    <row r="31" spans="1:17">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I30" s="67">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="K30" s="122"/>
+    </row>
+    <row r="31" spans="1:18">
       <c r="A31" s="112"/>
       <c r="B31" s="62" t="s">
         <v>413</v>
@@ -5800,12 +5971,15 @@
         <v>0</v>
       </c>
       <c r="H31" s="63">
-        <f t="shared" ref="H31:H38" si="6">SUM(C31:G31)</f>
-        <v>0</v>
-      </c>
-      <c r="J31" s="122"/>
-    </row>
-    <row r="32" spans="1:17">
+        <v>0</v>
+      </c>
+      <c r="I31" s="63">
+        <f>SUM(C31:H31)</f>
+        <v>0</v>
+      </c>
+      <c r="K31" s="122"/>
+    </row>
+    <row r="32" spans="1:18">
       <c r="A32" s="112"/>
       <c r="B32" s="62" t="s">
         <v>52</v>
@@ -5826,11 +6000,14 @@
         <v>0</v>
       </c>
       <c r="H32" s="88">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I32" s="88">
+        <f>SUM(C32:H32)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" s="112"/>
       <c r="B33" s="62" t="s">
         <v>14</v>
@@ -5851,11 +6028,14 @@
         <v>0</v>
       </c>
       <c r="H33" s="88">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I33" s="88">
+        <f>SUM(C33:H33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" s="112"/>
       <c r="B34" s="62" t="s">
         <v>53</v>
@@ -5876,11 +6056,14 @@
         <v>0</v>
       </c>
       <c r="H34" s="88">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I34" s="88">
+        <f>SUM(C34:H34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" s="112"/>
       <c r="B35" s="62" t="s">
         <v>54</v>
@@ -5901,11 +6084,14 @@
         <v>0</v>
       </c>
       <c r="H35" s="88">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I35" s="88">
+        <f>SUM(C35:H35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" s="112"/>
       <c r="B36" s="62" t="s">
         <v>55</v>
@@ -5926,11 +6112,14 @@
         <v>0</v>
       </c>
       <c r="H36" s="88">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I36" s="88">
+        <f>SUM(C36:H36)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37" s="112"/>
       <c r="B37" s="62" t="s">
         <v>56</v>
@@ -5951,11 +6140,14 @@
         <v>0</v>
       </c>
       <c r="H37" s="88">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10">
+        <v>0</v>
+      </c>
+      <c r="I37" s="88">
+        <f>SUM(C37:H37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" s="111">
         <v>8</v>
       </c>
@@ -5978,13 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="84">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J38" s="1"/>
-    </row>
-    <row r="39" spans="1:10" ht="15" customHeight="1" thickBot="1">
-      <c r="A39" s="147"/>
+        <v>0</v>
+      </c>
+      <c r="I38" s="84">
+        <f>SUM(C38:H38)</f>
+        <v>0</v>
+      </c>
+      <c r="K38" s="1"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" customHeight="1" thickBot="1">
+      <c r="A39" s="141"/>
       <c r="B39" s="41" t="s">
         <v>58</v>
       </c>
@@ -6009,25 +6204,29 @@
         <v>0</v>
       </c>
       <c r="H39" s="85">
-        <f>H30-H38-H36+H33+H35-H34-H32</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10">
+        <f>H30-H38-H36-H33+H35</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="85">
+        <f>I30-I38-I36+I33+I35-I34-I32</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" s="12"/>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:11">
       <c r="B41" s="12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:11">
       <c r="B44" s="127"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="74" orientation="landscape" r:id="rId1"/>
@@ -6040,7 +6239,7 @@
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="45.5546875" style="117" bestFit="1" customWidth="1"/>
@@ -6048,37 +6247,40 @@
     <col min="4" max="4" width="13.33203125" style="117" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.109375" style="117" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" style="117" customWidth="1"/>
-    <col min="7" max="7" width="14" style="117" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.88671875" style="117" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="117"/>
+    <col min="7" max="7" width="12.33203125" style="138" customWidth="1"/>
+    <col min="8" max="8" width="14" style="117" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="8.88671875" style="117" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" customHeight="1">
-      <c r="A1" s="138">
+    <row r="1" spans="1:9" ht="18" customHeight="1">
+      <c r="A1" s="142">
         <f>Summary!B1</f>
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="E1" s="139"/>
-      <c r="F1" s="139"/>
-      <c r="G1" s="139"/>
-      <c r="H1" s="118"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.6" customHeight="1">
-      <c r="A2" s="140" t="s">
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="118"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.6" customHeight="1">
+      <c r="A2" s="144" t="s">
         <v>415</v>
       </c>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="118"/>
-    </row>
-    <row r="3" spans="1:8" ht="18" customHeight="1" thickBot="1">
+      <c r="B2" s="143"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="118"/>
+    </row>
+    <row r="3" spans="1:9" ht="18" customHeight="1" thickBot="1">
       <c r="A3" s="50"/>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
@@ -6086,9 +6288,10 @@
       <c r="E3" s="42"/>
       <c r="F3" s="42"/>
       <c r="G3" s="42"/>
-      <c r="H3" s="118"/>
-    </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" thickBot="1">
+      <c r="H3" s="42"/>
+      <c r="I3" s="118"/>
+    </row>
+    <row r="4" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A4" s="51" t="s">
         <v>0</v>
       </c>
@@ -6112,13 +6315,17 @@
         <f>Summary!G4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="131" t="str">
+      <c r="G4" s="131">
         <f>Summary!H4</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="131" t="str">
+        <f>Summary!I4</f>
         <v>Total</v>
       </c>
-      <c r="H4" s="37"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I4" s="37"/>
+    </row>
+    <row r="5" spans="1:9" ht="14.4" customHeight="1">
       <c r="A5" s="52" t="s">
         <v>122</v>
       </c>
@@ -6128,9 +6335,10 @@
       <c r="E5" s="38"/>
       <c r="F5" s="43"/>
       <c r="G5" s="43"/>
-      <c r="H5" s="118"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H5" s="43"/>
+      <c r="I5" s="118"/>
+    </row>
+    <row r="6" spans="1:9" ht="14.4" customHeight="1">
       <c r="A6" s="49" t="s">
         <v>123</v>
       </c>
@@ -6154,13 +6362,17 @@
         <f>Cashflow!G5+Cashflow!G6+Cashflow!G9-Cashflow!G8-Cashflow!G29</f>
         <v>0</v>
       </c>
-      <c r="G6" s="92">
-        <f>SUM(B6:F6)</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="118"/>
-    </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" thickBot="1">
+      <c r="G6" s="88">
+        <f>Cashflow!H5+Cashflow!H6+Cashflow!H9-Cashflow!H8-Cashflow!H29</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="92">
+        <f>SUM(B6:G6)</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="118"/>
+    </row>
+    <row r="7" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A7" s="49" t="s">
         <v>124</v>
       </c>
@@ -6184,18 +6396,22 @@
         <f>Cashflow!G7</f>
         <v>0</v>
       </c>
-      <c r="G7" s="92">
-        <f>SUM(B7:F7)</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="118"/>
-    </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" thickBot="1">
+      <c r="G7" s="89">
+        <f>Cashflow!H7</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="92">
+        <f>SUM(B7:G7)</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="118"/>
+    </row>
+    <row r="8" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A8" s="53" t="s">
         <v>125</v>
       </c>
       <c r="B8" s="93">
-        <f t="shared" ref="B8:G8" si="0">B6+B7</f>
+        <f t="shared" ref="B8:H8" si="0">B6+B7</f>
         <v>0</v>
       </c>
       <c r="C8" s="93">
@@ -6214,13 +6430,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G8" s="94">
+      <c r="G8" s="93">
+        <f t="shared" ref="G8" si="1">G6+G7</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="94">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="118"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I8" s="118"/>
+    </row>
+    <row r="9" spans="1:9" ht="14.4" customHeight="1">
       <c r="A9" s="49"/>
       <c r="B9" s="89"/>
       <c r="C9" s="89"/>
@@ -6228,9 +6448,10 @@
       <c r="E9" s="89"/>
       <c r="F9" s="90"/>
       <c r="G9" s="90"/>
-      <c r="H9" s="118"/>
-    </row>
-    <row r="10" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H9" s="90"/>
+      <c r="I9" s="118"/>
+    </row>
+    <row r="10" spans="1:9" ht="14.4" customHeight="1">
       <c r="A10" s="54" t="s">
         <v>126</v>
       </c>
@@ -6254,23 +6475,28 @@
         <f>Cashflow!G11</f>
         <v>0</v>
       </c>
-      <c r="G10" s="92">
-        <f>SUM(B10:F10)</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="118"/>
-    </row>
-    <row r="11" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G10" s="89">
+        <f>Cashflow!H11</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="92">
+        <f>SUM(B10:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="118"/>
+    </row>
+    <row r="11" spans="1:9" ht="14.4" customHeight="1">
       <c r="A11" s="49"/>
       <c r="B11" s="89"/>
       <c r="C11" s="89"/>
       <c r="D11" s="89"/>
       <c r="E11" s="89"/>
       <c r="F11" s="90"/>
-      <c r="G11" s="91"/>
-      <c r="H11" s="118"/>
-    </row>
-    <row r="12" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G11" s="90"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="118"/>
+    </row>
+    <row r="12" spans="1:9" ht="14.4" customHeight="1">
       <c r="A12" s="54" t="s">
         <v>127</v>
       </c>
@@ -6294,23 +6520,28 @@
         <f>Cashflow!G21</f>
         <v>0</v>
       </c>
-      <c r="G12" s="92">
-        <f>SUM(B12:F12)</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="118"/>
-    </row>
-    <row r="13" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G12" s="89">
+        <f>Cashflow!H21</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="92">
+        <f>SUM(B12:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="118"/>
+    </row>
+    <row r="13" spans="1:9" ht="14.4" customHeight="1">
       <c r="A13" s="49"/>
       <c r="B13" s="89"/>
       <c r="C13" s="89"/>
       <c r="D13" s="89"/>
       <c r="E13" s="89"/>
       <c r="F13" s="90"/>
-      <c r="G13" s="91"/>
-      <c r="H13" s="118"/>
-    </row>
-    <row r="14" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G13" s="90"/>
+      <c r="H13" s="91"/>
+      <c r="I13" s="118"/>
+    </row>
+    <row r="14" spans="1:9" ht="14.4" customHeight="1">
       <c r="A14" s="54" t="s">
         <v>128</v>
       </c>
@@ -6334,23 +6565,28 @@
         <f>Cashflow!G18</f>
         <v>0</v>
       </c>
-      <c r="G14" s="92">
-        <f>SUM(B14:F14)</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="118"/>
-    </row>
-    <row r="15" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G14" s="89">
+        <f>Cashflow!H18</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="92">
+        <f>SUM(B14:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="118"/>
+    </row>
+    <row r="15" spans="1:9" ht="14.4" customHeight="1">
       <c r="A15" s="49"/>
       <c r="B15" s="89"/>
       <c r="C15" s="89"/>
       <c r="D15" s="89"/>
       <c r="E15" s="89"/>
       <c r="F15" s="90"/>
-      <c r="G15" s="91"/>
-      <c r="H15" s="118"/>
-    </row>
-    <row r="16" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G15" s="90"/>
+      <c r="H15" s="91"/>
+      <c r="I15" s="118"/>
+    </row>
+    <row r="16" spans="1:9" ht="14.4" customHeight="1">
       <c r="A16" s="54" t="s">
         <v>129</v>
       </c>
@@ -6374,13 +6610,17 @@
         <f>Cashflow!G13</f>
         <v>0</v>
       </c>
-      <c r="G16" s="92">
-        <f>SUM(B16:F16)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="118"/>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" thickBot="1">
+      <c r="G16" s="89">
+        <f>Cashflow!H13</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="92">
+        <f>SUM(B16:G16)</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="118"/>
+    </row>
+    <row r="17" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A17" s="49"/>
       <c r="B17" s="89"/>
       <c r="C17" s="89"/>
@@ -6388,39 +6628,44 @@
       <c r="E17" s="89"/>
       <c r="F17" s="90"/>
       <c r="G17" s="90"/>
-      <c r="H17" s="118"/>
-    </row>
-    <row r="18" spans="1:8" ht="14.4" customHeight="1" thickBot="1">
+      <c r="H17" s="90"/>
+      <c r="I17" s="118"/>
+    </row>
+    <row r="18" spans="1:9" ht="14.4" customHeight="1" thickBot="1">
       <c r="A18" s="55" t="s">
         <v>130</v>
       </c>
       <c r="B18" s="93">
-        <f t="shared" ref="B18:G18" si="1">B8-B10-B12-B14-B16</f>
+        <f t="shared" ref="B18:H18" si="2">B8-B10-B12-B14-B16</f>
         <v>0</v>
       </c>
       <c r="C18" s="93">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="D18" s="93">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="E18" s="93">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F18" s="93">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G18" s="94">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H18" s="118"/>
-    </row>
-    <row r="19" spans="1:8" ht="15" customHeight="1" thickBot="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="93">
+        <f t="shared" ref="G18" si="3">G8-G10-G12-G14-G16</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="94">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="118"/>
+    </row>
+    <row r="19" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A19" s="56" t="s">
         <v>131</v>
       </c>
@@ -6444,178 +6689,200 @@
         <f>IFERROR(F18/F8,0)</f>
         <v>0</v>
       </c>
-      <c r="G19" s="45" t="e">
-        <f>G18/G8</f>
+      <c r="G19" s="44">
+        <f>IFERROR(G18/G8,0)</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="45" t="e">
+        <f>H18/H8</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H19" s="118"/>
-    </row>
-    <row r="20" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I19" s="118"/>
+    </row>
+    <row r="20" spans="1:9" ht="14.4" customHeight="1">
       <c r="B20" s="118"/>
       <c r="C20" s="118"/>
       <c r="D20" s="118"/>
       <c r="E20" s="118"/>
       <c r="F20" s="118"/>
-      <c r="G20" s="118"/>
+      <c r="G20" s="139"/>
       <c r="H20" s="118"/>
-    </row>
-    <row r="21" spans="1:8" ht="17.399999999999999" customHeight="1">
+      <c r="I20" s="118"/>
+    </row>
+    <row r="21" spans="1:9" ht="17.399999999999999" customHeight="1">
       <c r="B21" s="132"/>
       <c r="C21" s="132"/>
       <c r="D21" s="132"/>
       <c r="E21" s="132"/>
       <c r="F21" s="132"/>
       <c r="G21" s="132"/>
-      <c r="H21" s="118"/>
-    </row>
-    <row r="22" spans="1:8" ht="19.2" customHeight="1">
+      <c r="H21" s="132"/>
+      <c r="I21" s="118"/>
+    </row>
+    <row r="22" spans="1:9" ht="19.2" customHeight="1">
       <c r="B22" s="132"/>
       <c r="C22" s="132"/>
       <c r="D22" s="132"/>
       <c r="E22" s="132"/>
       <c r="F22" s="132"/>
       <c r="G22" s="132"/>
-      <c r="H22" s="118"/>
-    </row>
-    <row r="23" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H22" s="132"/>
+      <c r="I22" s="118"/>
+    </row>
+    <row r="23" spans="1:9" ht="14.4" customHeight="1">
       <c r="B23" s="132"/>
       <c r="C23" s="132"/>
       <c r="D23" s="132"/>
       <c r="E23" s="132"/>
       <c r="F23" s="132"/>
       <c r="G23" s="132"/>
-      <c r="H23" s="118"/>
-    </row>
-    <row r="24" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H23" s="132"/>
+      <c r="I23" s="118"/>
+    </row>
+    <row r="24" spans="1:9" ht="14.4" customHeight="1">
       <c r="B24" s="118"/>
       <c r="C24" s="118"/>
       <c r="D24" s="118"/>
       <c r="E24" s="118"/>
       <c r="F24" s="118"/>
-      <c r="G24" s="118"/>
+      <c r="G24" s="139"/>
       <c r="H24" s="118"/>
-    </row>
-    <row r="25" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I24" s="118"/>
+    </row>
+    <row r="25" spans="1:9" ht="14.4" customHeight="1">
       <c r="B25" s="132"/>
       <c r="C25" s="132"/>
       <c r="D25" s="132"/>
       <c r="E25" s="132"/>
       <c r="F25" s="132"/>
       <c r="G25" s="132"/>
-      <c r="H25" s="118"/>
-    </row>
-    <row r="26" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H25" s="132"/>
+      <c r="I25" s="118"/>
+    </row>
+    <row r="26" spans="1:9" ht="14.4" customHeight="1">
       <c r="B26" s="118"/>
       <c r="C26" s="118"/>
       <c r="D26" s="118"/>
       <c r="E26" s="118"/>
       <c r="F26" s="118"/>
-      <c r="G26" s="118"/>
+      <c r="G26" s="139"/>
       <c r="H26" s="118"/>
-    </row>
-    <row r="27" spans="1:8" ht="8.4" customHeight="1">
+      <c r="I26" s="118"/>
+    </row>
+    <row r="27" spans="1:9" ht="8.4" customHeight="1">
       <c r="B27" s="118"/>
       <c r="C27" s="118"/>
       <c r="D27" s="118"/>
       <c r="E27" s="118"/>
       <c r="F27" s="118"/>
-      <c r="G27" s="118"/>
+      <c r="G27" s="139"/>
       <c r="H27" s="118"/>
-    </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1">
+      <c r="I27" s="118"/>
+    </row>
+    <row r="28" spans="1:9" ht="15" customHeight="1">
       <c r="B28" s="118"/>
       <c r="C28" s="118"/>
       <c r="D28" s="118"/>
       <c r="E28" s="118"/>
       <c r="F28" s="118"/>
-      <c r="G28" s="118"/>
+      <c r="G28" s="139"/>
       <c r="H28" s="118"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.6" customHeight="1">
+      <c r="I28" s="118"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.6" customHeight="1">
       <c r="B29" s="118"/>
       <c r="C29" s="118"/>
       <c r="D29" s="118"/>
       <c r="E29" s="118"/>
       <c r="F29" s="118"/>
-      <c r="G29" s="118"/>
+      <c r="G29" s="139"/>
       <c r="H29" s="118"/>
-    </row>
-    <row r="30" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I29" s="118"/>
+    </row>
+    <row r="30" spans="1:9" ht="14.4" customHeight="1">
       <c r="B30" s="118"/>
       <c r="C30" s="118"/>
       <c r="D30" s="118"/>
       <c r="E30" s="118"/>
       <c r="F30" s="118"/>
-      <c r="G30" s="118"/>
+      <c r="G30" s="139"/>
       <c r="H30" s="118"/>
-    </row>
-    <row r="31" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I30" s="118"/>
+    </row>
+    <row r="31" spans="1:9" ht="14.4" customHeight="1">
       <c r="B31" s="118"/>
       <c r="C31" s="118"/>
       <c r="D31" s="118"/>
       <c r="E31" s="118"/>
       <c r="F31" s="118"/>
-      <c r="G31" s="118"/>
+      <c r="G31" s="139"/>
       <c r="H31" s="118"/>
-    </row>
-    <row r="32" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I31" s="118"/>
+    </row>
+    <row r="32" spans="1:9" ht="14.4" customHeight="1">
       <c r="B32" s="118"/>
       <c r="C32" s="118"/>
       <c r="D32" s="118"/>
       <c r="E32" s="118"/>
       <c r="F32" s="118"/>
-      <c r="G32" s="118"/>
+      <c r="G32" s="139"/>
       <c r="H32" s="118"/>
-    </row>
-    <row r="33" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I32" s="118"/>
+    </row>
+    <row r="33" spans="2:9" ht="14.4" customHeight="1">
       <c r="B33" s="118"/>
       <c r="C33" s="118"/>
       <c r="D33" s="118"/>
       <c r="E33" s="118"/>
       <c r="F33" s="118"/>
-      <c r="G33" s="118"/>
+      <c r="G33" s="139"/>
       <c r="H33" s="118"/>
-    </row>
-    <row r="34" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I33" s="118"/>
+    </row>
+    <row r="34" spans="2:9" ht="14.4" customHeight="1">
       <c r="B34" s="118"/>
       <c r="C34" s="118"/>
       <c r="D34" s="118"/>
       <c r="E34" s="118"/>
       <c r="F34" s="118"/>
-      <c r="G34" s="118"/>
+      <c r="G34" s="139"/>
       <c r="H34" s="118"/>
-    </row>
-    <row r="35" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I34" s="118"/>
+    </row>
+    <row r="35" spans="2:9" ht="14.4" customHeight="1">
       <c r="B35" s="118"/>
       <c r="C35" s="118"/>
       <c r="D35" s="118"/>
       <c r="E35" s="118"/>
       <c r="F35" s="118"/>
-      <c r="G35" s="118"/>
+      <c r="G35" s="139"/>
       <c r="H35" s="118"/>
-    </row>
-    <row r="36" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I35" s="118"/>
+    </row>
+    <row r="36" spans="2:9" ht="14.4" customHeight="1">
       <c r="B36" s="118"/>
       <c r="C36" s="118"/>
       <c r="D36" s="118"/>
       <c r="E36" s="118"/>
       <c r="F36" s="118"/>
-      <c r="G36" s="118"/>
+      <c r="G36" s="139"/>
       <c r="H36" s="118"/>
-    </row>
-    <row r="37" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I36" s="118"/>
+    </row>
+    <row r="37" spans="2:9" ht="14.4" customHeight="1">
       <c r="B37" s="118"/>
       <c r="C37" s="118"/>
       <c r="D37" s="118"/>
       <c r="E37" s="118"/>
       <c r="F37" s="118"/>
-      <c r="G37" s="118"/>
+      <c r="G37" s="139"/>
       <c r="H37" s="118"/>
+      <c r="I37" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -6628,7 +6895,7 @@
   <sheetPr codeName="Sheet5">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="46.21875" style="117" customWidth="1"/>
@@ -6636,47 +6903,51 @@
     <col min="4" max="4" width="13.33203125" style="117" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.109375" style="117" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" style="117" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" style="117" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.88671875" style="117" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="117"/>
+    <col min="7" max="7" width="12.6640625" style="138" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="117" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="8.88671875" style="117" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="117"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.4" customHeight="1">
-      <c r="A1" s="138">
+    <row r="1" spans="1:9" ht="14.4" customHeight="1">
+      <c r="A1" s="142">
         <f>Summary!B1</f>
         <v>0</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="E1" s="139"/>
-      <c r="F1" s="139"/>
-      <c r="G1" s="139"/>
-      <c r="H1" s="36"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.6" customHeight="1">
-      <c r="A2" s="140" t="s">
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="36"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.6" customHeight="1">
+      <c r="A2" s="144" t="s">
         <v>416</v>
       </c>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="118"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" thickBot="1">
+      <c r="B2" s="143"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="118"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="118"/>
       <c r="B3" s="118"/>
       <c r="C3" s="118"/>
       <c r="D3" s="118"/>
       <c r="E3" s="118"/>
       <c r="F3" s="118"/>
-      <c r="G3" s="118"/>
+      <c r="G3" s="139"/>
       <c r="H3" s="118"/>
-    </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" thickBot="1">
+      <c r="I3" s="118"/>
+    </row>
+    <row r="4" spans="1:9" ht="15" customHeight="1" thickBot="1">
       <c r="A4" s="57" t="s">
         <v>0</v>
       </c>
@@ -6700,13 +6971,17 @@
         <f>Summary!G4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="133" t="str">
+      <c r="G4" s="133">
         <f>Summary!H4</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="133" t="str">
+        <f>Summary!I4</f>
         <v>Total</v>
       </c>
-      <c r="H4" s="37"/>
-    </row>
-    <row r="5" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I4" s="37"/>
+    </row>
+    <row r="5" spans="1:9" ht="14.4" customHeight="1">
       <c r="A5" s="48" t="s">
         <v>132</v>
       </c>
@@ -6716,9 +6991,10 @@
       <c r="E5" s="38"/>
       <c r="F5" s="38"/>
       <c r="G5" s="38"/>
-      <c r="H5" s="118"/>
-    </row>
-    <row r="6" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H5" s="38"/>
+      <c r="I5" s="118"/>
+    </row>
+    <row r="6" spans="1:9" ht="14.4" customHeight="1">
       <c r="A6" s="38" t="s">
         <v>133</v>
       </c>
@@ -6743,12 +7019,16 @@
         <v>0</v>
       </c>
       <c r="G6" s="86">
-        <f>SUM(B6:F6)</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="118"/>
-    </row>
-    <row r="7" spans="1:8" ht="14.4" customHeight="1">
+        <f>Cashflow!H10</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="86">
+        <f>SUM(B6:G6)</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="118"/>
+    </row>
+    <row r="7" spans="1:9" ht="14.4" customHeight="1">
       <c r="A7" s="38" t="s">
         <v>134</v>
       </c>
@@ -6757,18 +7037,19 @@
       <c r="D7" s="86"/>
       <c r="E7" s="86"/>
       <c r="F7" s="86"/>
-      <c r="G7" s="86">
-        <f>SUM(B7:F7)</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="118"/>
-    </row>
-    <row r="8" spans="1:8" ht="14.4" customHeight="1">
+      <c r="G7" s="86"/>
+      <c r="H7" s="86">
+        <f>SUM(B7:G7)</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="118"/>
+    </row>
+    <row r="8" spans="1:9" ht="14.4" customHeight="1">
       <c r="A8" s="47" t="s">
         <v>58</v>
       </c>
       <c r="B8" s="87">
-        <f t="shared" ref="B8:G8" si="0">B7-B6</f>
+        <f t="shared" ref="B8:H8" si="0">B7-B6</f>
         <v>0</v>
       </c>
       <c r="C8" s="87">
@@ -6788,12 +7069,16 @@
         <v>0</v>
       </c>
       <c r="G8" s="87">
+        <f t="shared" ref="G8" si="1">G7-G6</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="118"/>
-    </row>
-    <row r="9" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I8" s="118"/>
+    </row>
+    <row r="9" spans="1:9" ht="14.4" customHeight="1">
       <c r="A9" s="38"/>
       <c r="B9" s="39">
         <f>IFERROR(B8/B6,)</f>
@@ -6819,9 +7104,13 @@
         <f>IFERROR(G8/G6,0)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="118"/>
-    </row>
-    <row r="10" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H9" s="39">
+        <f>IFERROR(H8/H6,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="118"/>
+    </row>
+    <row r="10" spans="1:9" ht="14.4" customHeight="1">
       <c r="A10" s="38"/>
       <c r="B10" s="40"/>
       <c r="C10" s="40"/>
@@ -6829,9 +7118,10 @@
       <c r="E10" s="40"/>
       <c r="F10" s="40"/>
       <c r="G10" s="40"/>
-      <c r="H10" s="118"/>
-    </row>
-    <row r="11" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H10" s="40"/>
+      <c r="I10" s="118"/>
+    </row>
+    <row r="11" spans="1:9" ht="14.4" customHeight="1">
       <c r="A11" s="48" t="s">
         <v>135</v>
       </c>
@@ -6841,9 +7131,10 @@
       <c r="E11" s="134"/>
       <c r="F11" s="134"/>
       <c r="G11" s="134"/>
-      <c r="H11" s="118"/>
-    </row>
-    <row r="12" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H11" s="134"/>
+      <c r="I11" s="118"/>
+    </row>
+    <row r="12" spans="1:9" ht="14.4" customHeight="1">
       <c r="A12" s="38" t="s">
         <v>136</v>
       </c>
@@ -6863,12 +7154,15 @@
         <v>0</v>
       </c>
       <c r="G12" s="86">
-        <f>SUM(B12:F12)</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="118"/>
-    </row>
-    <row r="13" spans="1:8" ht="14.4" customHeight="1">
+        <v>0</v>
+      </c>
+      <c r="H12" s="86">
+        <f>SUM(B12:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="118"/>
+    </row>
+    <row r="13" spans="1:9" ht="14.4" customHeight="1">
       <c r="A13" s="38" t="s">
         <v>137</v>
       </c>
@@ -6888,12 +7182,15 @@
         <v>0</v>
       </c>
       <c r="G13" s="86">
-        <f>SUM(B13:F13)</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="118"/>
-    </row>
-    <row r="14" spans="1:8" ht="14.4" customHeight="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="86">
+        <f>SUM(B13:G13)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="118"/>
+    </row>
+    <row r="14" spans="1:9" ht="14.4" customHeight="1">
       <c r="A14" s="38"/>
       <c r="B14" s="86"/>
       <c r="C14" s="86"/>
@@ -6901,9 +7198,10 @@
       <c r="E14" s="86"/>
       <c r="F14" s="86"/>
       <c r="G14" s="86"/>
-      <c r="H14" s="118"/>
-    </row>
-    <row r="15" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H14" s="86"/>
+      <c r="I14" s="118"/>
+    </row>
+    <row r="15" spans="1:9" ht="14.4" customHeight="1">
       <c r="A15" s="38"/>
       <c r="B15" s="62"/>
       <c r="C15" s="62"/>
@@ -6911,9 +7209,10 @@
       <c r="E15" s="62"/>
       <c r="F15" s="62"/>
       <c r="G15" s="62"/>
-      <c r="H15" s="118"/>
-    </row>
-    <row r="16" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H15" s="62"/>
+      <c r="I15" s="118"/>
+    </row>
+    <row r="16" spans="1:9" ht="14.4" customHeight="1">
       <c r="A16" s="48" t="s">
         <v>138</v>
       </c>
@@ -6923,9 +7222,10 @@
       <c r="E16" s="62"/>
       <c r="F16" s="62"/>
       <c r="G16" s="62"/>
-      <c r="H16" s="118"/>
-    </row>
-    <row r="17" spans="1:8" ht="14.4" customHeight="1">
+      <c r="H16" s="62"/>
+      <c r="I16" s="118"/>
+    </row>
+    <row r="17" spans="1:9" ht="14.4" customHeight="1">
       <c r="A17" s="38" t="s">
         <v>139</v>
       </c>
@@ -6950,12 +7250,16 @@
         <v>0</v>
       </c>
       <c r="G17" s="86">
-        <f t="shared" ref="G17:G22" si="1">SUM(B17:F17)</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="118"/>
-    </row>
-    <row r="18" spans="1:8" ht="14.4" customHeight="1">
+        <f>Cashflow!H30</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="86">
+        <f>SUM(B17:G17)</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="118"/>
+    </row>
+    <row r="18" spans="1:9" ht="14.4" customHeight="1">
       <c r="A18" s="38" t="s">
         <v>140</v>
       </c>
@@ -6980,12 +7284,16 @@
         <v>0</v>
       </c>
       <c r="G18" s="86">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H18" s="118"/>
-    </row>
-    <row r="19" spans="1:8" ht="14.4" customHeight="1">
+        <f>Cashflow!H36</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="86">
+        <f>SUM(B18:G18)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="118"/>
+    </row>
+    <row r="19" spans="1:9" ht="14.4" customHeight="1">
       <c r="A19" s="38" t="s">
         <v>141</v>
       </c>
@@ -7010,12 +7318,16 @@
         <v>0</v>
       </c>
       <c r="G19" s="86">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H19" s="118"/>
-    </row>
-    <row r="20" spans="1:8" ht="14.4" customHeight="1">
+        <f>Cashflow!H34</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="86">
+        <f>SUM(B19:G19)</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="118"/>
+    </row>
+    <row r="20" spans="1:9" ht="14.4" customHeight="1">
       <c r="A20" s="38" t="s">
         <v>142</v>
       </c>
@@ -7039,12 +7351,15 @@
         <v>0</v>
       </c>
       <c r="G20" s="86">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H20" s="118"/>
-    </row>
-    <row r="21" spans="1:8" ht="14.4" customHeight="1">
+        <v>0</v>
+      </c>
+      <c r="H20" s="86">
+        <f>SUM(B20:G20)</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="118"/>
+    </row>
+    <row r="21" spans="1:9" ht="14.4" customHeight="1">
       <c r="A21" s="38" t="s">
         <v>143</v>
       </c>
@@ -7069,12 +7384,16 @@
         <v>0</v>
       </c>
       <c r="G21" s="86">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H21" s="118"/>
-    </row>
-    <row r="22" spans="1:8" ht="17.399999999999999" customHeight="1">
+        <f>Cashflow!H35</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="86">
+        <f>SUM(B21:G21)</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="118"/>
+    </row>
+    <row r="22" spans="1:9" ht="17.399999999999999" customHeight="1">
       <c r="A22" s="38" t="s">
         <v>144</v>
       </c>
@@ -7099,12 +7418,16 @@
         <v>0</v>
       </c>
       <c r="G22" s="86">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H22" s="118"/>
-    </row>
-    <row r="23" spans="1:8" ht="19.2" customHeight="1" thickBot="1">
+        <f>Cashflow!H38</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="86">
+        <f>SUM(B22:G22)</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="118"/>
+    </row>
+    <row r="23" spans="1:9" ht="19.2" customHeight="1" thickBot="1">
       <c r="A23" s="58" t="s">
         <v>58</v>
       </c>
@@ -7129,22 +7452,27 @@
         <v>0</v>
       </c>
       <c r="G23" s="41">
-        <f>G17-G22-G18+G20-G19</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="118"/>
-    </row>
-    <row r="24" spans="1:8" ht="14.4" customHeight="1">
+        <f>G17-G22-G18+G21</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="41">
+        <f>H17-H22-H18+H20-H19</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="118"/>
+    </row>
+    <row r="24" spans="1:9" ht="14.4" customHeight="1">
       <c r="A24" s="118"/>
       <c r="B24" s="118"/>
       <c r="C24" s="118"/>
       <c r="D24" s="118"/>
       <c r="E24" s="118"/>
       <c r="F24" s="118"/>
-      <c r="G24" s="118"/>
+      <c r="G24" s="139"/>
       <c r="H24" s="118"/>
-    </row>
-    <row r="25" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I24" s="118"/>
+    </row>
+    <row r="25" spans="1:9" ht="14.4" customHeight="1">
       <c r="A25" s="12" t="s">
         <v>145</v>
       </c>
@@ -7153,132 +7481,146 @@
       <c r="D25" s="118"/>
       <c r="E25" s="118"/>
       <c r="F25" s="118"/>
-      <c r="G25" s="118"/>
+      <c r="G25" s="139"/>
       <c r="H25" s="118"/>
-    </row>
-    <row r="26" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I25" s="118"/>
+    </row>
+    <row r="26" spans="1:9" ht="14.4" customHeight="1">
       <c r="A26" s="118"/>
       <c r="B26" s="118"/>
       <c r="C26" s="118"/>
       <c r="D26" s="118"/>
       <c r="E26" s="118"/>
       <c r="F26" s="118"/>
-      <c r="G26" s="118"/>
+      <c r="G26" s="139"/>
       <c r="H26" s="118"/>
-    </row>
-    <row r="27" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I26" s="118"/>
+    </row>
+    <row r="27" spans="1:9" ht="14.4" customHeight="1">
       <c r="A27" s="118"/>
       <c r="B27" s="118"/>
       <c r="C27" s="118"/>
       <c r="D27" s="118"/>
       <c r="E27" s="118"/>
       <c r="F27" s="118"/>
-      <c r="G27" s="118"/>
+      <c r="G27" s="139"/>
       <c r="H27" s="118"/>
-    </row>
-    <row r="28" spans="1:8" ht="8.4" customHeight="1">
+      <c r="I27" s="118"/>
+    </row>
+    <row r="28" spans="1:9" ht="8.4" customHeight="1">
       <c r="B28" s="118"/>
       <c r="C28" s="118"/>
       <c r="D28" s="118"/>
       <c r="E28" s="118"/>
       <c r="F28" s="118"/>
-      <c r="G28" s="118"/>
+      <c r="G28" s="139"/>
       <c r="H28" s="118"/>
-    </row>
-    <row r="29" spans="1:8" ht="15" customHeight="1">
+      <c r="I28" s="118"/>
+    </row>
+    <row r="29" spans="1:9" ht="15" customHeight="1">
       <c r="B29" s="118"/>
       <c r="C29" s="118"/>
       <c r="D29" s="118"/>
       <c r="E29" s="118"/>
       <c r="F29" s="118"/>
-      <c r="G29" s="118"/>
+      <c r="G29" s="139"/>
       <c r="H29" s="118"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.6" customHeight="1">
+      <c r="I29" s="118"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.6" customHeight="1">
       <c r="B30" s="118"/>
       <c r="C30" s="118"/>
       <c r="D30" s="118"/>
       <c r="E30" s="118"/>
       <c r="F30" s="118"/>
-      <c r="G30" s="118"/>
+      <c r="G30" s="139"/>
       <c r="H30" s="118"/>
-    </row>
-    <row r="31" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I30" s="118"/>
+    </row>
+    <row r="31" spans="1:9" ht="14.4" customHeight="1">
       <c r="B31" s="118"/>
       <c r="C31" s="118"/>
       <c r="D31" s="118"/>
       <c r="E31" s="118"/>
       <c r="F31" s="118"/>
-      <c r="G31" s="118"/>
+      <c r="G31" s="139"/>
       <c r="H31" s="118"/>
-    </row>
-    <row r="32" spans="1:8" ht="14.4" customHeight="1">
+      <c r="I31" s="118"/>
+    </row>
+    <row r="32" spans="1:9" ht="14.4" customHeight="1">
       <c r="B32" s="118"/>
       <c r="C32" s="118"/>
       <c r="D32" s="118"/>
       <c r="E32" s="118"/>
       <c r="F32" s="118"/>
-      <c r="G32" s="118"/>
+      <c r="G32" s="139"/>
       <c r="H32" s="118"/>
-    </row>
-    <row r="33" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I32" s="118"/>
+    </row>
+    <row r="33" spans="2:9" ht="14.4" customHeight="1">
       <c r="B33" s="118"/>
       <c r="C33" s="118"/>
       <c r="D33" s="118"/>
       <c r="E33" s="118"/>
       <c r="F33" s="118"/>
-      <c r="G33" s="118"/>
+      <c r="G33" s="139"/>
       <c r="H33" s="118"/>
-    </row>
-    <row r="34" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I33" s="118"/>
+    </row>
+    <row r="34" spans="2:9" ht="14.4" customHeight="1">
       <c r="B34" s="118"/>
       <c r="C34" s="118"/>
       <c r="D34" s="118"/>
       <c r="E34" s="118"/>
       <c r="F34" s="118"/>
-      <c r="G34" s="118"/>
+      <c r="G34" s="139"/>
       <c r="H34" s="118"/>
-    </row>
-    <row r="35" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I34" s="118"/>
+    </row>
+    <row r="35" spans="2:9" ht="14.4" customHeight="1">
       <c r="B35" s="118"/>
       <c r="C35" s="118"/>
       <c r="D35" s="118"/>
       <c r="E35" s="118"/>
       <c r="F35" s="118"/>
-      <c r="G35" s="118"/>
+      <c r="G35" s="139"/>
       <c r="H35" s="118"/>
-    </row>
-    <row r="36" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I35" s="118"/>
+    </row>
+    <row r="36" spans="2:9" ht="14.4" customHeight="1">
       <c r="B36" s="118"/>
       <c r="C36" s="118"/>
       <c r="D36" s="118"/>
       <c r="E36" s="118"/>
       <c r="F36" s="118"/>
-      <c r="G36" s="118"/>
+      <c r="G36" s="139"/>
       <c r="H36" s="118"/>
-    </row>
-    <row r="37" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I36" s="118"/>
+    </row>
+    <row r="37" spans="2:9" ht="14.4" customHeight="1">
       <c r="B37" s="118"/>
       <c r="C37" s="118"/>
       <c r="D37" s="118"/>
       <c r="E37" s="118"/>
       <c r="F37" s="118"/>
-      <c r="G37" s="118"/>
+      <c r="G37" s="139"/>
       <c r="H37" s="118"/>
-    </row>
-    <row r="38" spans="2:8" ht="14.4" customHeight="1">
+      <c r="I37" s="118"/>
+    </row>
+    <row r="38" spans="2:9" ht="14.4" customHeight="1">
       <c r="B38" s="118"/>
       <c r="C38" s="118"/>
       <c r="D38" s="118"/>
       <c r="E38" s="118"/>
       <c r="F38" s="118"/>
-      <c r="G38" s="118"/>
+      <c r="G38" s="139"/>
       <c r="H38" s="118"/>
+      <c r="I38" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix: add 6th week template support for Zpay and Paytm, fix date parsing and Errno 22 in Zomato Pay processing
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Varun\Desktop\Backup AutoRecons\Zomato Auto recons - Copy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74524162-0DFC-487B-9D16-2F3633219BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366D220A-5B22-452F-B1FF-429DC5A00BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="882" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="882" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -2316,6 +2316,12 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2338,12 +2344,6 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -2910,37 +2910,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="15" customHeight="1">
-      <c r="B1" s="142"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="143"/>
+      <c r="B1" s="144"/>
+      <c r="C1" s="145"/>
+      <c r="D1" s="145"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="145"/>
+      <c r="H1" s="145"/>
+      <c r="I1" s="145"/>
       <c r="J1" s="6"/>
     </row>
     <row r="2" spans="2:10" ht="16.5" customHeight="1">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="146" t="s">
         <v>417</v>
       </c>
-      <c r="C2" s="143"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="143"/>
-      <c r="F2" s="143"/>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
-      <c r="I2" s="143"/>
+      <c r="C2" s="145"/>
+      <c r="D2" s="145"/>
+      <c r="E2" s="145"/>
+      <c r="F2" s="145"/>
+      <c r="G2" s="145"/>
+      <c r="H2" s="145"/>
+      <c r="I2" s="145"/>
     </row>
     <row r="3" spans="2:10" ht="12" customHeight="1" thickBot="1">
-      <c r="B3" s="145"/>
-      <c r="C3" s="143"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="143"/>
-      <c r="F3" s="143"/>
-      <c r="G3" s="143"/>
-      <c r="H3" s="143"/>
-      <c r="I3" s="143"/>
+      <c r="B3" s="147"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="145"/>
+      <c r="F3" s="145"/>
+      <c r="G3" s="145"/>
+      <c r="H3" s="145"/>
+      <c r="I3" s="145"/>
     </row>
     <row r="4" spans="2:10" ht="15" customHeight="1" thickBot="1">
       <c r="B4" s="13" t="s">
@@ -2951,7 +2951,7 @@
       <c r="E4" s="120"/>
       <c r="F4" s="121"/>
       <c r="G4" s="120"/>
-      <c r="H4" s="151"/>
+      <c r="H4" s="142"/>
       <c r="I4" s="14" t="s">
         <v>1</v>
       </c>
@@ -2977,7 +2977,7 @@
       <c r="G6" s="99"/>
       <c r="H6" s="99"/>
       <c r="I6" s="96">
-        <f>SUM(C6:G6)</f>
+        <f>SUM(C6:H6)</f>
         <v>0</v>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       <c r="E15" s="99"/>
       <c r="F15" s="101"/>
       <c r="G15" s="102"/>
-      <c r="H15" s="152"/>
+      <c r="H15" s="143"/>
       <c r="I15" s="99"/>
     </row>
     <row r="16" spans="2:10" ht="14.4" customHeight="1">
@@ -5029,35 +5029,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18" customHeight="1">
-      <c r="A1" s="150">
+      <c r="A1" s="152">
         <f>Summary!B1</f>
         <v>0</v>
       </c>
-      <c r="B1" s="147"/>
-      <c r="C1" s="148"/>
-      <c r="D1" s="148"/>
-      <c r="E1" s="149"/>
-      <c r="F1" s="149"/>
-      <c r="G1" s="149"/>
-      <c r="H1" s="149"/>
-      <c r="I1" s="147"/>
+      <c r="B1" s="149"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="151"/>
+      <c r="F1" s="151"/>
+      <c r="G1" s="151"/>
+      <c r="H1" s="151"/>
+      <c r="I1" s="149"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
     </row>
     <row r="2" spans="1:18" ht="15.6" customHeight="1">
-      <c r="A2" s="146" t="s">
+      <c r="A2" s="148" t="s">
         <v>414</v>
       </c>
-      <c r="B2" s="147"/>
-      <c r="C2" s="148"/>
-      <c r="D2" s="148"/>
-      <c r="E2" s="149"/>
-      <c r="F2" s="149"/>
-      <c r="G2" s="149"/>
-      <c r="H2" s="149"/>
-      <c r="I2" s="147"/>
+      <c r="B2" s="149"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="149"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="46"/>
@@ -5507,27 +5507,27 @@
         <v>35</v>
       </c>
       <c r="C18" s="67">
-        <f>SUM(C19:C20)</f>
+        <f t="shared" ref="C18:H18" si="3">SUM(C19:C20)</f>
         <v>0</v>
       </c>
       <c r="D18" s="67">
-        <f>SUM(D19:D20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="E18" s="67">
-        <f>SUM(E19:E20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F18" s="67">
-        <f>SUM(F19:F20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G18" s="67">
-        <f>SUM(G19:G20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H18" s="67">
-        <f>SUM(H19:H20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I18" s="68">
@@ -5657,31 +5657,31 @@
         <v>41</v>
       </c>
       <c r="C21" s="67">
-        <f t="shared" ref="C21:I21" si="3">C22+C23+C24</f>
+        <f t="shared" ref="C21:I21" si="4">C22+C23+C24</f>
         <v>0</v>
       </c>
       <c r="D21" s="67">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="E21" s="68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="F21" s="68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G21" s="68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H21" s="68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I21" s="68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="M21" s="117" t="s">
@@ -5803,31 +5803,31 @@
         <v>46</v>
       </c>
       <c r="C25" s="67">
-        <f t="shared" ref="C25:I25" si="4">C10-C11-C18-C21-C13-C29</f>
+        <f t="shared" ref="C25:I25" si="5">C10-C11-C18-C21-C13-C29</f>
         <v>0</v>
       </c>
       <c r="D25" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="E25" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="F25" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G25" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H25" s="67">
-        <f t="shared" ref="H25" si="5">H10-H11-H18-H21-H13-H29</f>
+        <f t="shared" ref="H25" si="6">H10-H11-H18-H21-H13-H29</f>
         <v>0</v>
       </c>
       <c r="I25" s="67">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -5837,31 +5837,31 @@
         <v>47</v>
       </c>
       <c r="C26" s="67">
-        <f t="shared" ref="C26:I26" si="6">SUM(C27:C29)</f>
+        <f t="shared" ref="C26:I26" si="7">SUM(C27:C29)</f>
         <v>0</v>
       </c>
       <c r="D26" s="67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="E26" s="67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="F26" s="67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G26" s="67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="H26" s="67">
-        <f t="shared" ref="H26" si="7">SUM(H27:H29)</f>
+        <f t="shared" ref="H26" si="8">SUM(H27:H29)</f>
         <v>0</v>
       </c>
       <c r="I26" s="67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -5925,27 +5925,27 @@
         <v>0</v>
       </c>
       <c r="D30" s="67">
-        <f t="shared" ref="D30:I30" si="8">D25-D27-D28-D34</f>
+        <f t="shared" ref="D30:I30" si="9">D25-D27-D28-D34</f>
         <v>0</v>
       </c>
       <c r="E30" s="67">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F30" s="67">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="G30" s="67">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="H30" s="67">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="I30" s="67">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="K30" s="122"/>
@@ -5974,7 +5974,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="63">
-        <f>SUM(C31:H31)</f>
+        <f t="shared" ref="I31:I38" si="10">SUM(C31:H31)</f>
         <v>0</v>
       </c>
       <c r="K31" s="122"/>
@@ -6003,7 +6003,7 @@
         <v>0</v>
       </c>
       <c r="I32" s="88">
-        <f>SUM(C32:H32)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -6031,7 +6031,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="88">
-        <f>SUM(C33:H33)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -6059,7 +6059,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="88">
-        <f>SUM(C34:H34)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -6087,7 +6087,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="88">
-        <f>SUM(C35:H35)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -6115,7 +6115,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="88">
-        <f>SUM(C36:H36)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="88">
-        <f>SUM(C37:H37)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
@@ -6173,7 +6173,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="84">
-        <f>SUM(C38:H38)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="K38" s="1"/>
@@ -6254,30 +6254,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18" customHeight="1">
-      <c r="A1" s="142">
+      <c r="A1" s="144">
         <f>Summary!B1</f>
         <v>0</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
+      <c r="B1" s="145"/>
+      <c r="C1" s="145"/>
+      <c r="D1" s="145"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="145"/>
+      <c r="H1" s="145"/>
       <c r="I1" s="118"/>
     </row>
     <row r="2" spans="1:9" ht="15.6" customHeight="1">
-      <c r="A2" s="144" t="s">
+      <c r="A2" s="146" t="s">
         <v>415</v>
       </c>
-      <c r="B2" s="143"/>
-      <c r="C2" s="143"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="143"/>
-      <c r="F2" s="143"/>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
+      <c r="B2" s="145"/>
+      <c r="C2" s="145"/>
+      <c r="D2" s="145"/>
+      <c r="E2" s="145"/>
+      <c r="F2" s="145"/>
+      <c r="G2" s="145"/>
+      <c r="H2" s="145"/>
       <c r="I2" s="118"/>
     </row>
     <row r="3" spans="1:9" ht="18" customHeight="1" thickBot="1">
@@ -6670,27 +6670,27 @@
         <v>131</v>
       </c>
       <c r="B19" s="44">
-        <f>IFERROR(B18/B8,0)</f>
+        <f t="shared" ref="B19:G19" si="4">IFERROR(B18/B8,0)</f>
         <v>0</v>
       </c>
       <c r="C19" s="44">
-        <f>IFERROR(C18/C8,0)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="D19" s="44">
-        <f>IFERROR(D18/D8,0)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="E19" s="44">
-        <f>IFERROR(E18/E8,0)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="F19" s="44">
-        <f>IFERROR(F18/F8,0)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G19" s="44">
-        <f>IFERROR(G18/G8,0)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H19" s="45" t="e">
@@ -6910,30 +6910,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="14.4" customHeight="1">
-      <c r="A1" s="142">
+      <c r="A1" s="144">
         <f>Summary!B1</f>
         <v>0</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
+      <c r="B1" s="145"/>
+      <c r="C1" s="145"/>
+      <c r="D1" s="145"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="145"/>
+      <c r="H1" s="145"/>
       <c r="I1" s="36"/>
     </row>
     <row r="2" spans="1:9" ht="15.6" customHeight="1">
-      <c r="A2" s="144" t="s">
+      <c r="A2" s="146" t="s">
         <v>416</v>
       </c>
-      <c r="B2" s="143"/>
-      <c r="C2" s="143"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="143"/>
-      <c r="F2" s="143"/>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
+      <c r="B2" s="145"/>
+      <c r="C2" s="145"/>
+      <c r="D2" s="145"/>
+      <c r="E2" s="145"/>
+      <c r="F2" s="145"/>
+      <c r="G2" s="145"/>
+      <c r="H2" s="145"/>
       <c r="I2" s="118"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" thickBot="1">
@@ -7085,27 +7085,27 @@
         <v>0</v>
       </c>
       <c r="C9" s="39">
-        <f>IFERROR(C8/C6,0)</f>
+        <f t="shared" ref="C9:H9" si="2">IFERROR(C8/C6,0)</f>
         <v>0</v>
       </c>
       <c r="D9" s="39">
-        <f>IFERROR(D8/D6,0)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="E9" s="39">
-        <f>IFERROR(E8/E6,0)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="F9" s="39">
-        <f>IFERROR(F8/F6,0)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G9" s="39">
-        <f>IFERROR(G8/G6,0)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="H9" s="39">
-        <f>IFERROR(H8/H6,0)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I9" s="118"/>
@@ -7254,7 +7254,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="86">
-        <f>SUM(B17:G17)</f>
+        <f t="shared" ref="H17:H22" si="3">SUM(B17:G17)</f>
         <v>0</v>
       </c>
       <c r="I17" s="118"/>
@@ -7288,7 +7288,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="86">
-        <f>SUM(B18:G18)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I18" s="118"/>
@@ -7322,7 +7322,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="86">
-        <f>SUM(B19:G19)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I19" s="118"/>
@@ -7354,7 +7354,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="86">
-        <f>SUM(B20:G20)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I20" s="118"/>
@@ -7388,7 +7388,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="86">
-        <f>SUM(B21:G21)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I21" s="118"/>
@@ -7422,7 +7422,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="86">
-        <f>SUM(B22:G22)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I22" s="118"/>

</xml_diff>